<commit_message>
VERSIÓN 7 FINAL INCLUYE TODA LA INFORMACIÓN
</commit_message>
<xml_diff>
--- a/CONSULTA INVENTARIO.xlsx
+++ b/CONSULTA INVENTARIO.xlsx
@@ -137,17 +137,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DETALLE" displayName="DETALLE" ref="A1:H3" headerRowCount="1">
-  <autoFilter ref="A1:H3"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DETALLE" displayName="DETALLE" ref="A1:I3" headerRowCount="1">
+  <autoFilter ref="A1:I3"/>
+  <tableColumns count="9">
     <tableColumn id="1" name="ENUMBER"/>
     <tableColumn id="2" name="N° PAREJA"/>
     <tableColumn id="3" name="MESA"/>
     <tableColumn id="4" name="LISTADO"/>
     <tableColumn id="5" name="UBICACIÓN A CONTAR"/>
-    <tableColumn id="6" name="HORARIO DE COLACIÓN"/>
+    <tableColumn id="6" name="HORARIO BREAK MAÑANA"/>
     <tableColumn id="7" name="HORARIO DE ALMUERZO"/>
-    <tableColumn id="8" name="ACTIVO"/>
+    <tableColumn id="8" name="HORARIO BREAK TARDE"/>
+    <tableColumn id="9" name="ACTIVO"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -442,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -450,9 +451,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,7 +485,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>HORARIO DE COLACIÓN</t>
+          <t>HORARIO BREAK MAÑANA</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -492,6 +494,11 @@
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HORARIO BREAK TARDE</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
@@ -535,6 +542,11 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>16:00 - 16:15</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
@@ -576,6 +588,11 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>16:00 - 16:15</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>

</xml_diff>